<commit_message>
Update TS2#79 via Streamlit
</commit_message>
<xml_diff>
--- a/TS2_mapping.xlsx
+++ b/TS2_mapping.xlsx
@@ -3762,7 +3762,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3772,7 +3772,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>無資料</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update TS2#90 via Streamlit
</commit_message>
<xml_diff>
--- a/TS2_mapping.xlsx
+++ b/TS2_mapping.xlsx
@@ -4224,7 +4224,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -4234,7 +4234,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>無資料</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update TS2#90 Mapping via Tab3
</commit_message>
<xml_diff>
--- a/TS2_mapping.xlsx
+++ b/TS2_mapping.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update TS2#1 Mapping via Tab3
</commit_message>
<xml_diff>
--- a/TS2_mapping.xlsx
+++ b/TS2_mapping.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update TS2_mapping.xlsx via Streamlit
</commit_message>
<xml_diff>
--- a/TS2_mapping.xlsx
+++ b/TS2_mapping.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>